<commit_message>
Flat-price coupons (BHOLEKRIPA → ₹10) + phone country-code auto-detect
Excel gains a Flat_Price_INR column; parser emits richer manifest
({type, value}). JS handles both percent and flat_inr coupons.
Phone inputs strip non-digits and auto-route a typed/pasted "+CC"
prefix to the country dropdown, keeping only the local number.
</commit_message>
<xml_diff>
--- a/Discount.xlsx
+++ b/Discount.xlsx
@@ -1,81 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/AshishKumar.Soni/Downloads/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BA8139D0-1D55-F949-A964-C47E2366BC99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="680" windowWidth="28040" windowHeight="16940" xr2:uid="{2C227B1C-0945-2148-BEBF-2BB0041C2E90}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="680" yWindow="680" windowWidth="28040" windowHeight="16940" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
-  <si>
-    <t>Discount_Coupon</t>
-  </si>
-  <si>
-    <t>Discount_Percentage</t>
-  </si>
-  <si>
-    <t>100OFF</t>
-  </si>
-  <si>
-    <t>50OFF</t>
-  </si>
-  <si>
-    <t>20OFF</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -94,23 +53,82 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -430,44 +448,73 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{149E38B8-CBD3-E445-87B5-950B320984CF}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col width="15.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="18.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Discount_Coupon</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Discount_Percentage</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Flat_Price_INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>100OFF</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="2">
-        <v>1</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>50OFF</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>0.5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="2">
-        <v>0.5</v>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>20OFF</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>0.2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="2">
-        <v>0.2</v>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BHOLEKRIPA</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Coupon catalog: keep only 20OFF + BHOLEKRIPA; hide BHOLEKRIPA from Offers
- Removed 100OFF and 50OFF rows from Discount.xlsx
- Regenerated coupons-manifest.js (2 entries now)
- BHOLEKRIPA still works when typed manually but is filtered out
  of the public Offers modal via INTERNAL_COUPONS allowlist
</commit_message>
<xml_diff>
--- a/Discount.xlsx
+++ b/Discount.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="15.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -480,40 +480,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>100OFF</t>
+          <t>20OFF</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>50OFF</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>20OFF</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
           <t>BHOLEKRIPA</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C3" t="n">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add WIN30: 30% off, Windows Softwares only
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Discount.xlsx
+++ b/Discount.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="15.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -512,6 +512,21 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>WIN30</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Validity column to coupons; expire codes past their date
- Discount.xlsx: new "Validity" column (date format) for per-coupon expiry
- update-coupons.py: parse Excel serial / ISO date in column E, emit `validity`
- index.html: reject expired codes at apply time with "has expired" message
  and hide them from the public Offers modal

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Discount.xlsx
+++ b/Discount.xlsx
@@ -1,89 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/AshishKumar.Soni/Downloads/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0B1D250-E688-514D-A218-2BF7984D7B90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="680" windowWidth="28040" windowHeight="16920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="680" yWindow="680" windowWidth="28040" windowHeight="16920" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
-  <si>
-    <t>Discount_Coupon</t>
-  </si>
-  <si>
-    <t>Discount_Percentage</t>
-  </si>
-  <si>
-    <t>Applies_To</t>
-  </si>
-  <si>
-    <t>both</t>
-  </si>
-  <si>
-    <t>BHOLEKRIPA</t>
-  </si>
-  <si>
-    <t>windows</t>
-  </si>
-  <si>
-    <t>macbook</t>
-  </si>
-  <si>
-    <t>Internal_Discount_Percentage</t>
-  </si>
-  <si>
-    <t>QSZERO</t>
-  </si>
-  <si>
-    <t>FLAT90</t>
-  </si>
-  <si>
-    <t>WIN10</t>
-  </si>
-  <si>
-    <t>MAC15</t>
-  </si>
-  <si>
-    <t>QS50PC</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
+  <fonts count="2">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -101,24 +54,84 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -438,94 +451,142 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
+    <col width="15.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="18.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="26" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Discount_Coupon</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Discount_Percentage</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Internal_Discount_Percentage</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Applies_To</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Validity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BHOLEKRIPA</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>WIN10</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MAC15</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>macbook</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>QSZERO</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="2">
-        <v>0.99</v>
-      </c>
-      <c r="D2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3">
-        <v>0.1</v>
-      </c>
-      <c r="D3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="2">
-        <v>0.15</v>
-      </c>
-      <c r="D4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="2">
-        <v>1</v>
-      </c>
-      <c r="D5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="2">
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>FLAT90</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
         <v>0.9</v>
       </c>
-      <c r="D6" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="2">
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>QS50PC</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="D7" t="s">
-        <v>3</v>
-      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Set BHOLEKRIPA validity to 2026-06-12 for expiry testing
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Discount.xlsx
+++ b/Discount.xlsx
@@ -506,7 +506,9 @@
           <t>both</t>
         </is>
       </c>
-      <c r="E2" s="3" t="n"/>
+      <c r="E2" s="3" t="n">
+        <v>46185</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">

</xml_diff>

<commit_message>
Make tiered discount Excel-driven from Discount.xlsx
Add a "Tiers" sheet to Discount.xlsx (one row per platform: Off_Qty2/3/4,
Cap_Qty, Charge_Top_N, Cap_Off, Cap_Message) and have update-coupons.py
parse it into window.TIERS alongside window.COUPONS. The parser now
resolves worksheets by name (workbook.xml + rels) instead of assuming
sheet1.xml, so sheet ordering no longer matters; it stays stdlib-only for
CI. index.html reads window.TIERS with a built-in fallback so older
manifests keep working. Output is forced to UTF-8/LF for consistency with
the CI (Linux) regeneration.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Discount.xlsx
+++ b/Discount.xlsx
@@ -1,98 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/AshishKumar.Soni/Downloads/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC21AAE3-AFD6-1148-BDA2-633EB99B4781}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="680" windowWidth="28040" windowHeight="16920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="680" yWindow="680" windowWidth="28040" windowHeight="16920" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tiers" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
-  <si>
-    <t>Discount_Coupon</t>
-  </si>
-  <si>
-    <t>Discount_Percentage</t>
-  </si>
-  <si>
-    <t>Internal_Discount_Percentage</t>
-  </si>
-  <si>
-    <t>Applies_To</t>
-  </si>
-  <si>
-    <t>Validity</t>
-  </si>
-  <si>
-    <t>BHOLEKRIPA</t>
-  </si>
-  <si>
-    <t>both</t>
-  </si>
-  <si>
-    <t>WIN10</t>
-  </si>
-  <si>
-    <t>windows</t>
-  </si>
-  <si>
-    <t>MAC15</t>
-  </si>
-  <si>
-    <t>macbook</t>
-  </si>
-  <si>
-    <t>QSZERO</t>
-  </si>
-  <si>
-    <t>FLAT90</t>
-  </si>
-  <si>
-    <t>QS50PC</t>
-  </si>
-  <si>
-    <t>QS25WL</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -111,24 +56,83 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -448,122 +452,290 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
+    <col width="15.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="18.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="26" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Discount_Coupon</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Discount_Percentage</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Internal_Discount_Percentage</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Applies_To</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Validity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BHOLEKRIPA</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>WIN10</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MAC15</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>macbook</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>QSZERO</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="2">
-        <v>0.99</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="3"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3">
-        <v>0.1</v>
-      </c>
-      <c r="D3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="3"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="2">
-        <v>0.15</v>
-      </c>
-      <c r="D4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="3"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="2">
-        <v>1</v>
-      </c>
-      <c r="D5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" s="3"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="2">
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>FLAT90</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
         <v>0.9</v>
       </c>
-      <c r="D6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" s="3"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="2">
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>QS50PC</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="D7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7" s="3">
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n">
         <v>46192</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" s="2">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>QS25WL</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
         <v>0.25</v>
       </c>
-      <c r="D8" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8" s="3">
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
         <v>46192</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Off_Qty2</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Off_Qty3</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Off_Qty4</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Cap_Qty</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Charge_Top_N</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Cap_Off</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Cap_Message</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>500</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>5 or more Softwares at Rs. 6000</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>macbook</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D3" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>5000</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>5 or more Softwares at Rs. 7500</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>